<commit_message>
Update indexed metadata workbook
</commit_message>
<xml_diff>
--- a/data/metadata/Quercus_metadata_with_index.xlsx
+++ b/data/metadata/Quercus_metadata_with_index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://missouribotanicalgarden.sharepoint.com/sites/IMLSNationalLeadershipGrant20232/Shared Documents/General/Manuscript/Quercus/data/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_093208354DD74F3DB7492A619882BDA412D04BB7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA188F56-6C08-1049-BC42-FB9895344E2A}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_093208354DD74F3DB7492A619882BDA412D04BB7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC0D66CD-150E-C04D-BDCD-58D373BCD9FA}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="500" windowWidth="34560" windowHeight="19600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6780" uniqueCount="1295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6800" uniqueCount="1302">
   <si>
     <t>x</t>
   </si>
@@ -3909,6 +3909,27 @@
   </si>
   <si>
     <t>AR/LA</t>
+  </si>
+  <si>
+    <t>Missouri</t>
+  </si>
+  <si>
+    <t>Saint Louis city</t>
+  </si>
+  <si>
+    <t>Small tree at the side gate of MOBOT</t>
+  </si>
+  <si>
+    <t>Big tree at the side gate of MOBOT</t>
+  </si>
+  <si>
+    <t>Big tree in Tower Grove Park, nearby farmer's market plaza</t>
+  </si>
+  <si>
+    <t>East of Central crossing</t>
+  </si>
+  <si>
+    <t>Intersection of Magnolia and 39th street</t>
   </si>
 </sst>
 </file>
@@ -3918,7 +3939,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss\ \U\T\C"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3936,8 +3957,14 @@
       <color theme="1"/>
       <name val="Calibri (Body)"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3947,6 +3974,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -3962,7 +3995,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3977,6 +4010,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4224,6 +4264,7 @@
     <col min="15" max="15" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.33203125" customWidth="1"/>
     <col min="19" max="19" width="12.6640625" customWidth="1"/>
+    <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="20.6640625" style="2" customWidth="1"/>
     <col min="26" max="26" width="17.6640625" customWidth="1"/>
     <col min="28" max="28" width="9" customWidth="1"/>
@@ -29762,7 +29803,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="257" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="257" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D257" t="s">
         <v>958</v>
       </c>
@@ -29786,7 +29827,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="258" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="258" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D258" t="s">
         <v>960</v>
       </c>
@@ -29810,7 +29851,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="259" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="259" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D259" t="s">
         <v>961</v>
       </c>
@@ -29834,7 +29875,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="260" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="260" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D260" t="s">
         <v>962</v>
       </c>
@@ -29867,7 +29908,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="261" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="261" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D261" t="s">
         <v>965</v>
       </c>
@@ -29894,7 +29935,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="262" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="262" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D262" t="s">
         <v>967</v>
       </c>
@@ -29927,7 +29968,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="263" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="263" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D263" t="s">
         <v>969</v>
       </c>
@@ -29960,7 +30001,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="264" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="264" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D264" t="s">
         <v>971</v>
       </c>
@@ -29987,7 +30028,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="265" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="265" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D265" t="s">
         <v>973</v>
       </c>
@@ -30018,7 +30059,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="266" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="266" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D266" t="s">
         <v>976</v>
       </c>
@@ -30049,7 +30090,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="267" spans="4:15" x14ac:dyDescent="0.2">
+    <row r="267" spans="4:32" x14ac:dyDescent="0.2">
       <c r="D267" t="s">
         <v>979</v>
       </c>
@@ -30081,141 +30122,206 @@
         <v>981</v>
       </c>
     </row>
-    <row r="268" spans="4:15" x14ac:dyDescent="0.2">
-      <c r="D268" t="s">
+    <row r="268" spans="4:32" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D268" s="8" t="s">
         <v>982</v>
       </c>
-      <c r="E268" t="s">
+      <c r="E268" s="8" t="s">
         <v>982</v>
       </c>
-      <c r="F268" t="s">
+      <c r="F268" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G268" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H268" t="s">
-        <v>48</v>
-      </c>
-      <c r="I268" t="s">
-        <v>48</v>
-      </c>
-      <c r="K268">
+      <c r="G268" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H268" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I268" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="K268" s="8">
         <v>49</v>
       </c>
-      <c r="L268" s="4" t="s">
+      <c r="L268" s="10" t="s">
         <v>983</v>
       </c>
-      <c r="M268" s="3"/>
-      <c r="N268" s="3"/>
-      <c r="O268" t="s">
+      <c r="M268" s="9"/>
+      <c r="N268" s="9"/>
+      <c r="O268" s="8" t="s">
         <v>941</v>
       </c>
-    </row>
-    <row r="269" spans="4:15" x14ac:dyDescent="0.2">
-      <c r="D269" t="s">
+      <c r="Q268" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="R268" s="12" t="s">
+        <v>1295</v>
+      </c>
+      <c r="S268" s="12" t="s">
+        <v>1296</v>
+      </c>
+      <c r="Y268" s="11"/>
+      <c r="AF268" s="12" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="269" spans="4:32" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D269" s="8" t="s">
         <v>984</v>
       </c>
-      <c r="E269" t="s">
+      <c r="E269" s="8" t="s">
         <v>984</v>
       </c>
-      <c r="F269" t="s">
+      <c r="F269" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G269" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H269" t="s">
-        <v>48</v>
-      </c>
-      <c r="I269" t="s">
-        <v>48</v>
-      </c>
-      <c r="K269">
+      <c r="G269" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H269" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I269" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="K269" s="8">
         <v>90.4</v>
       </c>
-      <c r="L269" s="4" t="s">
+      <c r="L269" s="10" t="s">
         <v>985</v>
       </c>
-      <c r="M269" s="3"/>
-      <c r="N269" s="3"/>
-      <c r="O269" t="s">
+      <c r="M269" s="9"/>
+      <c r="N269" s="9"/>
+      <c r="O269" s="8" t="s">
         <v>941</v>
       </c>
-    </row>
-    <row r="270" spans="4:15" x14ac:dyDescent="0.2">
-      <c r="D270" t="s">
+      <c r="Q269" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="R269" s="12" t="s">
+        <v>1295</v>
+      </c>
+      <c r="S269" s="12" t="s">
+        <v>1296</v>
+      </c>
+      <c r="Y269" s="11"/>
+      <c r="AF269" s="12" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="270" spans="4:32" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D270" s="8" t="s">
         <v>986</v>
       </c>
-      <c r="E270" t="s">
+      <c r="E270" s="8" t="s">
         <v>986</v>
       </c>
-      <c r="F270" t="s">
+      <c r="F270" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G270" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K270">
+      <c r="G270" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K270" s="8">
         <v>53</v>
       </c>
-      <c r="L270" s="4" t="s">
+      <c r="L270" s="10" t="s">
         <v>987</v>
       </c>
-      <c r="M270" s="3"/>
-      <c r="N270" s="3"/>
-      <c r="O270" t="s">
+      <c r="M270" s="9"/>
+      <c r="N270" s="9"/>
+      <c r="O270" s="8" t="s">
         <v>941</v>
       </c>
-    </row>
-    <row r="271" spans="4:15" x14ac:dyDescent="0.2">
-      <c r="D271" t="s">
+      <c r="Q270" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="R270" s="12" t="s">
+        <v>1295</v>
+      </c>
+      <c r="S270" s="12" t="s">
+        <v>1296</v>
+      </c>
+      <c r="Y270" s="11"/>
+      <c r="AF270" s="12" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="271" spans="4:32" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D271" s="8" t="s">
         <v>988</v>
       </c>
-      <c r="E271" t="s">
+      <c r="E271" s="8" t="s">
         <v>988</v>
       </c>
-      <c r="F271" t="s">
+      <c r="F271" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G271" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K271">
+      <c r="G271" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K271" s="8">
         <v>39.799999999999997</v>
       </c>
-      <c r="L271" s="4" t="s">
+      <c r="L271" s="10" t="s">
         <v>989</v>
       </c>
-      <c r="M271" s="3"/>
-      <c r="N271" s="3"/>
-      <c r="O271" t="s">
+      <c r="M271" s="9"/>
+      <c r="N271" s="9"/>
+      <c r="O271" s="8" t="s">
         <v>941</v>
       </c>
-    </row>
-    <row r="272" spans="4:15" x14ac:dyDescent="0.2">
-      <c r="D272" t="s">
+      <c r="Q271" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="R271" s="12" t="s">
+        <v>1295</v>
+      </c>
+      <c r="S271" s="12" t="s">
+        <v>1296</v>
+      </c>
+      <c r="Y271" s="11"/>
+      <c r="AF271" s="12" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="272" spans="4:32" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="D272" s="8" t="s">
         <v>990</v>
       </c>
-      <c r="E272" t="s">
+      <c r="E272" s="8" t="s">
         <v>990</v>
       </c>
-      <c r="F272" t="s">
+      <c r="F272" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G272" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K272">
+      <c r="G272" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K272" s="8">
         <v>70.8</v>
       </c>
-      <c r="L272" s="4" t="s">
+      <c r="L272" s="10" t="s">
         <v>991</v>
       </c>
-      <c r="M272" s="3"/>
-      <c r="N272" s="3"/>
-      <c r="O272" t="s">
+      <c r="M272" s="9"/>
+      <c r="N272" s="9"/>
+      <c r="O272" s="8" t="s">
         <v>941</v>
+      </c>
+      <c r="Q272" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="R272" s="12" t="s">
+        <v>1295</v>
+      </c>
+      <c r="S272" s="12" t="s">
+        <v>1296</v>
+      </c>
+      <c r="Y272" s="11"/>
+      <c r="AF272" s="12" t="s">
+        <v>1301</v>
       </c>
     </row>
     <row r="273" spans="4:15" x14ac:dyDescent="0.2">

</xml_diff>